<commit_message>
feat: flujos exportados y evidencias del taller
</commit_message>
<xml_diff>
--- a/robot_causaciones/datos/por_radicar.xlsx
+++ b/robot_causaciones/datos/por_radicar.xlsx
@@ -1,37 +1,125 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30606"/>
   <workbookPr/>
-  <workbookProtection/>
+  <xr:revisionPtr revIDLastSave="15" documentId="11_3003F0384A0A11C7A879F75EE173F286379506B9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{60D9F23E-A601-472C-9432-7495A1C71ABB}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="PorRadicar" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="PorRadicar" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
+  <si>
+    <t>IdLista</t>
+  </si>
+  <si>
+    <t>Factura</t>
+  </si>
+  <si>
+    <t>NIT</t>
+  </si>
+  <si>
+    <t>Proveedor</t>
+  </si>
+  <si>
+    <t>Valor</t>
+  </si>
+  <si>
+    <t>CentroCosto</t>
+  </si>
+  <si>
+    <t>FechaFactura</t>
+  </si>
+  <si>
+    <t>FE-20871</t>
+  </si>
+  <si>
+    <t>Empaques del Caribe S.A.S.</t>
+  </si>
+  <si>
+    <t>CC-100</t>
+  </si>
+  <si>
+    <t>ST-3307</t>
+  </si>
+  <si>
+    <t>Servicios Tecnológicos Andinos Ltda.</t>
+  </si>
+  <si>
+    <t>CC-300</t>
+  </si>
+  <si>
+    <t>MI-0077</t>
+  </si>
+  <si>
+    <t>Mantenimientos Industriales Ruiz S.A.S.</t>
+  </si>
+  <si>
+    <t>CC-200</t>
+  </si>
+  <si>
+    <t>PS-1188</t>
+  </si>
+  <si>
+    <t>Papelería y Suministros Central S.A.S.</t>
+  </si>
+  <si>
+    <t>Insumos Químicos del Valle S.A.S.</t>
+  </si>
+  <si>
+    <t>CC-400</t>
+  </si>
+  <si>
+    <t>TR-5530</t>
+  </si>
+  <si>
+    <t>Transportes Rápidos de Antioquia S.A.</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -49,98 +137,40 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PorRadicar" displayName="PorRadicar" ref="A1:G2" headerRowCount="1">
-  <autoFilter ref="A1:G2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="PorRadicar" displayName="PorRadicar" ref="A1:G8">
+  <autoFilter ref="A1:G8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="7">
-    <tableColumn id="1" name="IdLista"/>
-    <tableColumn id="2" name="Factura"/>
-    <tableColumn id="3" name="NIT"/>
-    <tableColumn id="4" name="Proveedor"/>
-    <tableColumn id="5" name="Valor"/>
-    <tableColumn id="6" name="CentroCosto"/>
-    <tableColumn id="7" name="FechaFactura"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="IdLista"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Factura"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="NIT"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Proveedor"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Valor"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="CentroCosto"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="FechaFactura"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -428,64 +458,182 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col min="1" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="4" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>IdLista</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Factura</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>NIT</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Proveedor</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Valor</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>CentroCosto</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>FechaFactura</t>
-        </is>
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3">
+        <v>900123456</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3">
+        <v>1850000</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" s="2">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4">
+        <v>830456789</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4">
+        <v>4200000</v>
+      </c>
+      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="2">
+        <v>46297</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5">
+        <v>900999001</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5">
+        <v>950000</v>
+      </c>
+      <c r="F5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="2">
+        <v>46297</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6">
+        <v>23</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6">
+        <v>860567890</v>
+      </c>
+      <c r="D6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6">
+        <v>620000</v>
+      </c>
+      <c r="F6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="2">
+        <v>46402</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7">
+        <v>901345678</v>
+      </c>
+      <c r="D7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7">
+        <v>2300000</v>
+      </c>
+      <c r="F7" t="s">
+        <v>19</v>
+      </c>
+      <c r="G7" s="2">
+        <v>46300</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8">
+        <v>19</v>
+      </c>
+      <c r="B8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8">
+        <v>800234567</v>
+      </c>
+      <c r="D8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8">
+        <v>6400000</v>
+      </c>
+      <c r="F8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G8" s="2">
+        <v>46295</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>